<commit_message>
Add Regression_Data sheet with 11 SPSS-ready predictor columns
Clean subset of Y + 10 predictors selected for multiple linear regression,
trimming dummy variables and individual Likert items.

https://claude.ai/code/session_01XW68jRwJoN62D7AQQcF2uU
</commit_message>
<xml_diff>
--- a/coded_survey_data.xlsx
+++ b/coded_survey_data.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Codebook" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Key" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Regression_Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Key" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -113,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -134,6 +135,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -19286,6 +19291,3937 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K112"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>MonthlyOnlineSpend_Y</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>MonthlyIncome</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>DisposableIncome</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>ShoppingFrequency</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>AvgPerPurchase</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>WhyShop_Avg</t>
+        </is>
+      </c>
+      <c r="I1" s="8" t="inlineStr">
+        <is>
+          <t>Influence_Avg</t>
+        </is>
+      </c>
+      <c r="J1" s="8" t="inlineStr">
+        <is>
+          <t>HoursOnline</t>
+        </is>
+      </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>SocialMediaDiscovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>125</v>
+      </c>
+      <c r="B3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>63</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>125</v>
+      </c>
+      <c r="B5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>63</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>125</v>
+      </c>
+      <c r="B7" t="n">
+        <v>29</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>88</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>125</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>125</v>
+      </c>
+      <c r="B11" t="n">
+        <v>19</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>63</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
+      <c r="F12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>175</v>
+      </c>
+      <c r="B13" t="n">
+        <v>22</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>88</v>
+      </c>
+      <c r="H13" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>175</v>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>225</v>
+      </c>
+      <c r="B15" t="n">
+        <v>23</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>125</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>175</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>175</v>
+      </c>
+      <c r="B17" t="n">
+        <v>23</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>88</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>125</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>75</v>
+      </c>
+      <c r="B19" t="n">
+        <v>26</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>63</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>33</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>75</v>
+      </c>
+      <c r="B21" t="n">
+        <v>26</v>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>63</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>75</v>
+      </c>
+      <c r="B23" t="n">
+        <v>22</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>63</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>75</v>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>63</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I25" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>75</v>
+      </c>
+      <c r="B27" t="n">
+        <v>22</v>
+      </c>
+      <c r="C27" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>63</v>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K28" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>75</v>
+      </c>
+      <c r="B29" t="n">
+        <v>25</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" t="n">
+        <v>63</v>
+      </c>
+      <c r="H29" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J30" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>75</v>
+      </c>
+      <c r="B31" t="n">
+        <v>21</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>63</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" t="n">
+        <v>22</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" t="n">
+        <v>88</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I34" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>25</v>
+      </c>
+      <c r="B35" t="n">
+        <v>23</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>63</v>
+      </c>
+      <c r="H35" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B36" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="I36" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>25</v>
+      </c>
+      <c r="B37" t="n">
+        <v>26</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>63</v>
+      </c>
+      <c r="H37" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I37" t="n">
+        <v>4</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B38" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I38" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J38" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K38" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>25</v>
+      </c>
+      <c r="B39" t="n">
+        <v>20</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>63</v>
+      </c>
+      <c r="H39" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I39" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K39" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B40" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C40" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>88</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I40" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J40" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K40" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>175</v>
+      </c>
+      <c r="B41" t="n">
+        <v>26</v>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>38</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="n">
+        <v>225</v>
+      </c>
+      <c r="B42" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C42" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I42" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K42" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>75</v>
+      </c>
+      <c r="B43" t="n">
+        <v>25</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" t="n">
+        <v>38</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I44" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K44" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>75</v>
+      </c>
+      <c r="B45" t="n">
+        <v>25</v>
+      </c>
+      <c r="C45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" t="n">
+        <v>38</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I45" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J45" t="n">
+        <v>2</v>
+      </c>
+      <c r="K45" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I46" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J46" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K46" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>75</v>
+      </c>
+      <c r="B47" t="n">
+        <v>30</v>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" t="n">
+        <v>38</v>
+      </c>
+      <c r="H47" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I47" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B48" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I48" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J48" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>75</v>
+      </c>
+      <c r="B49" t="n">
+        <v>23</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>38</v>
+      </c>
+      <c r="H49" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I50" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>75</v>
+      </c>
+      <c r="B51" t="n">
+        <v>28</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F51" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" t="n">
+        <v>38</v>
+      </c>
+      <c r="H51" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I51" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C52" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="9" t="inlineStr"/>
+      <c r="F52" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="I52" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>75</v>
+      </c>
+      <c r="B53" t="n">
+        <v>22</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G53" t="n">
+        <v>38</v>
+      </c>
+      <c r="H53" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J53" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B54" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I54" s="9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>75</v>
+      </c>
+      <c r="B55" t="n">
+        <v>24</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" t="n">
+        <v>38</v>
+      </c>
+      <c r="H55" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I55" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B56" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="C56" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I56" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>75</v>
+      </c>
+      <c r="B57" t="n">
+        <v>21</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>2</v>
+      </c>
+      <c r="G57" t="n">
+        <v>38</v>
+      </c>
+      <c r="H57" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I57" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J57" t="n">
+        <v>3</v>
+      </c>
+      <c r="K57" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C58" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H58" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I58" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>75</v>
+      </c>
+      <c r="B59" t="n">
+        <v>21</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" t="n">
+        <v>38</v>
+      </c>
+      <c r="H59" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I59" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J59" t="n">
+        <v>4</v>
+      </c>
+      <c r="K59" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B60" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="C60" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D60" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E60" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H60" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I60" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J60" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K60" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>75</v>
+      </c>
+      <c r="B61" t="n">
+        <v>27</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G61" t="n">
+        <v>12</v>
+      </c>
+      <c r="H61" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I61" t="n">
+        <v>4</v>
+      </c>
+      <c r="J61" t="n">
+        <v>3</v>
+      </c>
+      <c r="K61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C62" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H62" s="9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="I62" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J62" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K62" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>75</v>
+      </c>
+      <c r="B63" t="n">
+        <v>24</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>3</v>
+      </c>
+      <c r="G63" t="n">
+        <v>38</v>
+      </c>
+      <c r="H63" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I63" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J63" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B64" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="9" t="inlineStr"/>
+      <c r="F64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H64" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I64" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J64" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K64" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>75</v>
+      </c>
+      <c r="B65" t="n">
+        <v>26</v>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="n">
+        <v>38</v>
+      </c>
+      <c r="H65" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I65" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J65" t="n">
+        <v>3</v>
+      </c>
+      <c r="K65" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H66" s="9" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I66" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>75</v>
+      </c>
+      <c r="B67" t="n">
+        <v>21</v>
+      </c>
+      <c r="C67" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" t="n">
+        <v>12</v>
+      </c>
+      <c r="H67" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="I67" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2</v>
+      </c>
+      <c r="K67" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B68" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H68" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I68" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J68" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>25</v>
+      </c>
+      <c r="B69" t="n">
+        <v>26</v>
+      </c>
+      <c r="C69" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>2</v>
+      </c>
+      <c r="G69" t="n">
+        <v>12</v>
+      </c>
+      <c r="H69" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I69" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="J69" t="n">
+        <v>2</v>
+      </c>
+      <c r="K69" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H70" s="9" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="I70" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="J70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K70" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>25</v>
+      </c>
+      <c r="B71" t="n">
+        <v>23</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G71" t="n">
+        <v>12</v>
+      </c>
+      <c r="H71" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="I71" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J71" t="n">
+        <v>3</v>
+      </c>
+      <c r="K71" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B72" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H72" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I72" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J72" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K72" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>25</v>
+      </c>
+      <c r="B73" t="n">
+        <v>24</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="n">
+        <v>12</v>
+      </c>
+      <c r="H73" t="n">
+        <v>4</v>
+      </c>
+      <c r="I73" t="n">
+        <v>4</v>
+      </c>
+      <c r="J73" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B74" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C74" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D74" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H74" s="9" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="I74" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J74" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K74" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>25</v>
+      </c>
+      <c r="B75" t="n">
+        <v>40</v>
+      </c>
+      <c r="C75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" t="n">
+        <v>4</v>
+      </c>
+      <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="n">
+        <v>12</v>
+      </c>
+      <c r="H75" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I75" t="n">
+        <v>3</v>
+      </c>
+      <c r="J75" t="n">
+        <v>1</v>
+      </c>
+      <c r="K75" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B76" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C76" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I76" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J76" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>25</v>
+      </c>
+      <c r="B77" t="n">
+        <v>23</v>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" t="n">
+        <v>12</v>
+      </c>
+      <c r="H77" t="n">
+        <v>1</v>
+      </c>
+      <c r="I77" t="n">
+        <v>1</v>
+      </c>
+      <c r="J77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C78" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H78" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I78" s="9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J78" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K78" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>25</v>
+      </c>
+      <c r="B79" t="n">
+        <v>23</v>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2</v>
+      </c>
+      <c r="G79" t="n">
+        <v>38</v>
+      </c>
+      <c r="H79" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I79" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J79" t="n">
+        <v>3</v>
+      </c>
+      <c r="K79" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B80" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="C80" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H80" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I80" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J80" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K80" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>25</v>
+      </c>
+      <c r="B81" t="n">
+        <v>26</v>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" t="n">
+        <v>38</v>
+      </c>
+      <c r="H81" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I81" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J81" t="n">
+        <v>5</v>
+      </c>
+      <c r="K81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B82" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C82" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H82" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I82" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J82" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K82" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>25</v>
+      </c>
+      <c r="B83" t="n">
+        <v>31</v>
+      </c>
+      <c r="C83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" t="n">
+        <v>38</v>
+      </c>
+      <c r="H83" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I83" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="J83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K83" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B84" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C84" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H84" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I84" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J84" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K84" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>25</v>
+      </c>
+      <c r="B85" t="n">
+        <v>24</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>2</v>
+      </c>
+      <c r="G85" t="n">
+        <v>12</v>
+      </c>
+      <c r="H85" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I85" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J85" t="n">
+        <v>3</v>
+      </c>
+      <c r="K85" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B86" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C86" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D86" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H86" s="9" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="I86" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K86" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>25</v>
+      </c>
+      <c r="B87" t="n">
+        <v>22</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" t="n">
+        <v>12</v>
+      </c>
+      <c r="H87" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="I87" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J87" t="n">
+        <v>1</v>
+      </c>
+      <c r="K87" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B88" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C88" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D88" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E88" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H88" s="9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I88" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J88" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K88" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>25</v>
+      </c>
+      <c r="B89" t="n">
+        <v>24</v>
+      </c>
+      <c r="C89" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2</v>
+      </c>
+      <c r="G89" t="n">
+        <v>12</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4</v>
+      </c>
+      <c r="I89" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J89" t="n">
+        <v>1</v>
+      </c>
+      <c r="K89" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B90" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F90" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H90" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I90" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="J90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K90" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>25</v>
+      </c>
+      <c r="B91" t="n">
+        <v>23</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" t="n">
+        <v>12</v>
+      </c>
+      <c r="H91" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I91" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J91" t="n">
+        <v>2</v>
+      </c>
+      <c r="K91" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B92" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C92" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H92" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I92" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J92" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K92" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>25</v>
+      </c>
+      <c r="B93" t="n">
+        <v>24</v>
+      </c>
+      <c r="C93" t="n">
+        <v>2</v>
+      </c>
+      <c r="D93" t="n">
+        <v>2</v>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" t="n">
+        <v>38</v>
+      </c>
+      <c r="H93" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I93" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J93" t="n">
+        <v>3</v>
+      </c>
+      <c r="K93" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B94" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C94" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D94" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H94" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I94" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J94" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K94" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>25</v>
+      </c>
+      <c r="B95" t="n">
+        <v>23</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" t="n">
+        <v>38</v>
+      </c>
+      <c r="H95" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I95" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J95" t="n">
+        <v>4</v>
+      </c>
+      <c r="K95" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B96" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C96" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" s="9" t="inlineStr"/>
+      <c r="E96" s="9" t="inlineStr"/>
+      <c r="F96" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H96" s="9" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I96" s="9" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J96" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K96" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>25</v>
+      </c>
+      <c r="B97" t="n">
+        <v>22</v>
+      </c>
+      <c r="C97" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" t="n">
+        <v>12</v>
+      </c>
+      <c r="H97" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I97" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J97" t="n">
+        <v>4</v>
+      </c>
+      <c r="K97" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B98" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="C98" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H98" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I98" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J98" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K98" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>25</v>
+      </c>
+      <c r="B99" t="n">
+        <v>25</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="n">
+        <v>2</v>
+      </c>
+      <c r="G99" t="n">
+        <v>38</v>
+      </c>
+      <c r="H99" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I99" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J99" t="n">
+        <v>3</v>
+      </c>
+      <c r="K99" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B100" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C100" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H100" s="9" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I100" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J100" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K100" s="9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>25</v>
+      </c>
+      <c r="B101" t="n">
+        <v>22</v>
+      </c>
+      <c r="C101" t="n">
+        <v>2</v>
+      </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" t="n">
+        <v>38</v>
+      </c>
+      <c r="H101" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I101" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J101" t="n">
+        <v>3</v>
+      </c>
+      <c r="K101" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B102" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C102" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D102" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="9" t="inlineStr"/>
+      <c r="F102" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H102" s="9" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I102" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J102" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K102" s="9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>25</v>
+      </c>
+      <c r="B103" t="n">
+        <v>21</v>
+      </c>
+      <c r="C103" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1</v>
+      </c>
+      <c r="G103" t="n">
+        <v>38</v>
+      </c>
+      <c r="H103" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I103" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="J103" t="n">
+        <v>3</v>
+      </c>
+      <c r="K103" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B104" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C104" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D104" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G104" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H104" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I104" s="9" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J104" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K104" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>25</v>
+      </c>
+      <c r="B105" t="n">
+        <v>19</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" t="n">
+        <v>2</v>
+      </c>
+      <c r="F105" t="n">
+        <v>1</v>
+      </c>
+      <c r="G105" t="n">
+        <v>12</v>
+      </c>
+      <c r="H105" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I105" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J105" t="n">
+        <v>4</v>
+      </c>
+      <c r="K105" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B106" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="C106" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E106" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H106" s="9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I106" s="9" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="J106" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K106" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>25</v>
+      </c>
+      <c r="B107" t="n">
+        <v>22</v>
+      </c>
+      <c r="C107" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
+      <c r="E107" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" t="n">
+        <v>38</v>
+      </c>
+      <c r="H107" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I107" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J107" t="n">
+        <v>2</v>
+      </c>
+      <c r="K107" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B108" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="C108" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D108" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="H108" s="9" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I108" s="9" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J108" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K108" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>25</v>
+      </c>
+      <c r="B109" t="n">
+        <v>23</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" t="n">
+        <v>12</v>
+      </c>
+      <c r="H109" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="I109" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B110" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="C110" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D110" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G110" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H110" s="9" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I110" s="9" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="J110" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K110" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>25</v>
+      </c>
+      <c r="B111" t="n">
+        <v>19</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1</v>
+      </c>
+      <c r="G111" t="n">
+        <v>12</v>
+      </c>
+      <c r="H111" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3</v>
+      </c>
+      <c r="J111" t="n">
+        <v>4</v>
+      </c>
+      <c r="K111" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B112" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="C112" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D112" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G112" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H112" s="9" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I112" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J112" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K112" s="9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -19295,157 +23231,157 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Likert Scale Key (applies to all WhyShop_*, Influence_*, and Discourages_* columns)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="A3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Strongly Disagree</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Respondent strongly disagrees with the statement</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="A4" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Disagree</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Respondent disagrees with the statement</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="A5" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Respondent neither agrees nor disagrees</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Agree</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Respondent agrees with the statement</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Strongly Agree</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Respondent strongly agrees with the statement</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Average Column Key</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>WhyShop_Avg</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Orange</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Mean of 8 'Why do you shop online?' Likert items (1–5)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Influence_Avg</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Mean of 8 'What influences your purchase decisions?' Likert items (1–5)</t>
         </is>

</xml_diff>

<commit_message>
Replace nominal Situation with ordinal EmploymentLevel in Regression_Data
Situation (7 unordered nominal categories) is not valid for MLR. Replaced
with EmploymentLevel (ordinal 1-3): 1=Not earning, 2=Partially earning,
3=Fully earning. Full nominal coding preserved in the Data sheet.

https://claude.ai/code/session_01XW68jRwJoN62D7AQQcF2uU
</commit_message>
<xml_diff>
--- a/coded_survey_data.xlsx
+++ b/coded_survey_data.xlsx
@@ -18371,7 +18371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19277,6 +19277,23 @@
       <c r="C53" s="7" t="inlineStr">
         <is>
           <t>1=Never, 2=Rarely, 3=Sometimes, 4=Often, 5=Very Frequently</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>EmploymentLevel</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>Ordinal</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Regression_Data only. Collapsed from Situation. 1=Not earning (Student non-working / Unemployed / Stay-at-home), 2=Partially earning (Student working / Employed part-time), 3=Fully earning (Employed full-time / Self-employed)</t>
         </is>
       </c>
     </row>
@@ -19296,7 +19313,7 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
@@ -19320,7 +19337,7 @@
       </c>
       <c r="C1" s="8" t="inlineStr">
         <is>
-          <t>Situation</t>
+          <t>EmploymentLevel</t>
         </is>
       </c>
       <c r="D1" s="8" t="inlineStr">
@@ -19510,7 +19527,7 @@
         <v>28</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>2</v>
@@ -19650,7 +19667,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>5</v>
@@ -19819,7 +19836,7 @@
         <v>23</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>5</v>
@@ -19992,7 +20009,7 @@
         <v>33</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>2</v>
@@ -20237,7 +20254,7 @@
         <v>22</v>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
         <v>2</v>
@@ -20549,7 +20566,7 @@
         <v>22</v>
       </c>
       <c r="C36" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D36" s="9" t="n">
         <v>1</v>
@@ -20584,7 +20601,7 @@
         <v>26</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
         <v>2</v>
@@ -20934,7 +20951,7 @@
         <v>30</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
         <v>3</v>
@@ -21109,7 +21126,7 @@
         <v>26</v>
       </c>
       <c r="C52" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>1</v>
@@ -21317,7 +21334,7 @@
         <v>23</v>
       </c>
       <c r="C58" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D58" s="9" t="n">
         <v>2</v>
@@ -21872,7 +21889,7 @@
         <v>26</v>
       </c>
       <c r="C74" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D74" s="9" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Remove all non-dummy nominal variables from Data and Regression sheets
- Replaced Situation (nominal 7-cat) with EmploymentLevel (ordinal 1-3) throughout
- RelationshipStatus reclassified as Ordinal (1=Single to 4=Married, by commitment level)
- Only dummy variables (Income_*, Buy_*) remain as non-ordinal/scale

https://claude.ai/code/session_01XW68jRwJoN62D7AQQcF2uU
</commit_message>
<xml_diff>
--- a/coded_survey_data.xlsx
+++ b/coded_survey_data.xlsx
@@ -546,7 +546,7 @@
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Situation</t>
+          <t>EmploymentLevel</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1498,7 +1498,7 @@
         <v>28</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>4</v>
@@ -2130,7 +2130,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>1</v>
@@ -2914,7 +2914,7 @@
         <v>23</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
@@ -3702,7 +3702,7 @@
         <v>33</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>3</v>
@@ -4808,7 +4808,7 @@
         <v>22</v>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
         <v>3</v>
@@ -6227,7 +6227,7 @@
         <v>22</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>1</v>
@@ -6385,7 +6385,7 @@
         <v>26</v>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
         <v>2</v>
@@ -7965,7 +7965,7 @@
         <v>30</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
         <v>3</v>
@@ -8755,7 +8755,7 @@
         <v>26</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D52" s="4" t="n">
         <v>1</v>
@@ -9701,7 +9701,7 @@
         <v>23</v>
       </c>
       <c r="C58" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D58" s="4" t="n">
         <v>2</v>
@@ -12224,7 +12224,7 @@
         <v>26</v>
       </c>
       <c r="C74" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D74" s="4" t="n">
         <v>2</v>
@@ -18371,7 +18371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -18433,17 +18433,17 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Situation</t>
+          <t>EmploymentLevel</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Nominal</t>
+          <t>Ordinal</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>1=Student (non-working), 2=Student (working), 3=Employed full-time, 4=Employed part-time, 5=Self-employed, 6=Unemployed, 7=Stay-at-home</t>
+          <t>1=Not earning (Student non-working / Unemployed / Stay-at-home), 2=Partially earning (Student working / Employed part-time), 3=Fully earning (Employed full-time / Self-employed). Collapsed from 7-category employment question into ordered earning capacity levels.</t>
         </is>
       </c>
     </row>
@@ -18455,12 +18455,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Nominal</t>
+          <t>Ordinal</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>1=Single, 2=In a relationship, 3=Cohabiting, 4=Married; messy values normalised before coding</t>
+          <t>1=Single, 2=In a relationship, 3=Cohabiting, 4=Married. Treated as ordinal by increasing relationship commitment/stability; messy values normalised before coding.</t>
         </is>
       </c>
     </row>
@@ -19277,23 +19277,6 @@
       <c r="C53" s="7" t="inlineStr">
         <is>
           <t>1=Never, 2=Rarely, 3=Sometimes, 4=Often, 5=Very Frequently</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="inlineStr">
-        <is>
-          <t>EmploymentLevel</t>
-        </is>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>Ordinal</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Regression_Data only. Collapsed from Situation. 1=Not earning (Student non-working / Unemployed / Stay-at-home), 2=Partially earning (Student working / Employed part-time), 3=Fully earning (Employed full-time / Self-employed)</t>
         </is>
       </c>
     </row>

</xml_diff>